<commit_message>
Refactor auth controller, remove duplicate migration, and add evaluation metrics (precision, recall, specificity, f1-score) to K-NN testing
</commit_message>
<xml_diff>
--- a/public/training_data/data_training_v1.xlsx
+++ b/public/training_data/data_training_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\SIMPEL-5\public\training_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5667DFD-24A6-4CC4-B0C6-2238DE59411F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96422B95-09EE-4E35-97E3-60784EBFF781}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{14D7D6EB-D4B4-4E2B-8CF7-0BB7D653A469}"/>
   </bookViews>
@@ -2396,7 +2396,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2406,12 +2406,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2522,7 +2516,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>